<commit_message>
add guest page ans auth
</commit_message>
<xml_diff>
--- a/import/Tovar.xlsx
+++ b/import/Tovar.xlsx
@@ -1,30 +1,64 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Новая папка (2)\Пример\import\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arzam\OneDrive\Рабочий стол\exxx\import\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5CF7B47-7EAE-4251-B3AC-EC465D8543F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5640"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
+    <sheet name="Лист2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="164">
   <si>
     <t>Артикул</t>
   </si>
@@ -318,13 +352,211 @@
   </si>
   <si>
     <t>9.jpg</t>
+  </si>
+  <si>
+    <t>Тип товара</t>
+  </si>
+  <si>
+    <t>Единицы измерения</t>
+  </si>
+  <si>
+    <t>поставщик</t>
+  </si>
+  <si>
+    <t>категория товара</t>
+  </si>
+  <si>
+    <t>Роль сотрудника</t>
+  </si>
+  <si>
+    <t>ФИО</t>
+  </si>
+  <si>
+    <t>Логин</t>
+  </si>
+  <si>
+    <t>Пароль</t>
+  </si>
+  <si>
+    <t>Администратор</t>
+  </si>
+  <si>
+    <t>Никифорова Весения Николаевна</t>
+  </si>
+  <si>
+    <t>94d5ous@gmail.com</t>
+  </si>
+  <si>
+    <t>uzWC67</t>
+  </si>
+  <si>
+    <t>Сазонов Руслан Германович</t>
+  </si>
+  <si>
+    <t>uth4iz@mail.com</t>
+  </si>
+  <si>
+    <t>2L6KZG</t>
+  </si>
+  <si>
+    <t>Одинцов Серафим Артёмович</t>
+  </si>
+  <si>
+    <t>yzls62@outlook.com</t>
+  </si>
+  <si>
+    <t>JlFRCZ</t>
+  </si>
+  <si>
+    <t>Менеджер</t>
+  </si>
+  <si>
+    <t>Степанов Михаил Артёмович</t>
+  </si>
+  <si>
+    <t>1diph5e@tutanota.com</t>
+  </si>
+  <si>
+    <t>8ntwUp</t>
+  </si>
+  <si>
+    <t>Ворсин Петр Евгеньевич</t>
+  </si>
+  <si>
+    <t>tjde7c@yahoo.com</t>
+  </si>
+  <si>
+    <t>YOyhfR</t>
+  </si>
+  <si>
+    <t>Старикова Елена Павловна</t>
+  </si>
+  <si>
+    <t>wpmrc3do@tutanota.com</t>
+  </si>
+  <si>
+    <t>RSbvHv</t>
+  </si>
+  <si>
+    <t>Авторизированный клиент</t>
+  </si>
+  <si>
+    <t>Михайлюк Анна Вячеславовна</t>
+  </si>
+  <si>
+    <t>5d4zbu@tutanota.com</t>
+  </si>
+  <si>
+    <t>rwVDh9</t>
+  </si>
+  <si>
+    <t>Ситдикова Елена Анатольевна</t>
+  </si>
+  <si>
+    <t>ptec8ym@yahoo.com</t>
+  </si>
+  <si>
+    <t>LdNyos</t>
+  </si>
+  <si>
+    <t>1qz4kw@mail.com</t>
+  </si>
+  <si>
+    <t>gynQMT</t>
+  </si>
+  <si>
+    <t>4np6se@mail.com</t>
+  </si>
+  <si>
+    <t>AtnDjr</t>
+  </si>
+  <si>
+    <t>Роль</t>
+  </si>
+  <si>
+    <t>Фамилия</t>
+  </si>
+  <si>
+    <t>Имя</t>
+  </si>
+  <si>
+    <t>Отчество</t>
+  </si>
+  <si>
+    <t>Роли</t>
+  </si>
+  <si>
+    <t>Никифорова</t>
+  </si>
+  <si>
+    <t>Весения</t>
+  </si>
+  <si>
+    <t>Николаевна</t>
+  </si>
+  <si>
+    <t>Сазонов</t>
+  </si>
+  <si>
+    <t>Руслан</t>
+  </si>
+  <si>
+    <t>Германович</t>
+  </si>
+  <si>
+    <t>Одинцов</t>
+  </si>
+  <si>
+    <t>Серафим</t>
+  </si>
+  <si>
+    <t>Артёмович</t>
+  </si>
+  <si>
+    <t>Степанов</t>
+  </si>
+  <si>
+    <t>Михаил</t>
+  </si>
+  <si>
+    <t>Ворсин</t>
+  </si>
+  <si>
+    <t>Петр</t>
+  </si>
+  <si>
+    <t>Евгеньевич</t>
+  </si>
+  <si>
+    <t>Старикова</t>
+  </si>
+  <si>
+    <t>Елена</t>
+  </si>
+  <si>
+    <t>Павловна</t>
+  </si>
+  <si>
+    <t>Михайлюк</t>
+  </si>
+  <si>
+    <t>Анна</t>
+  </si>
+  <si>
+    <t>Вячеславовна</t>
+  </si>
+  <si>
+    <t>Ситдикова</t>
+  </si>
+  <si>
+    <t>Анатольевна</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="9">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -346,13 +578,62 @@
       <name val="Times Roman"/>
       <charset val="204"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -379,10 +660,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -390,11 +672,28 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -706,20 +1005,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K44"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:O75"/>
+  <sheetFormatPr defaultColWidth="11.25" defaultRowHeight="15.75"/>
   <cols>
-    <col min="2" max="2" width="16.69921875" customWidth="1"/>
-    <col min="3" max="3" width="21.69921875" customWidth="1"/>
-    <col min="5" max="5" width="21.296875" customWidth="1"/>
-    <col min="6" max="6" width="23.19921875" customWidth="1"/>
-    <col min="7" max="7" width="22.296875" customWidth="1"/>
+    <col min="2" max="2" width="16.75" customWidth="1"/>
+    <col min="3" max="3" width="21.75" customWidth="1"/>
+    <col min="5" max="5" width="21.25" customWidth="1"/>
+    <col min="6" max="6" width="23.25" customWidth="1"/>
+    <col min="7" max="7" width="22.25" customWidth="1"/>
     <col min="10" max="10" width="75" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="46.8">
+    <row r="1" spans="1:11" ht="47.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1777,7 +2076,7 @@
       <c r="J32" s="3"/>
       <c r="K32" s="3"/>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:15">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -1790,7 +2089,7 @@
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:15">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -1803,49 +2102,105 @@
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
     </row>
-    <row r="35" spans="1:11">
+    <row r="35" spans="1:15">
       <c r="A35" s="3"/>
-      <c r="B35" s="3"/>
+      <c r="B35" s="3" t="s">
+        <v>98</v>
+      </c>
       <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3"/>
+      <c r="E35" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>100</v>
+      </c>
       <c r="I35" s="3"/>
-      <c r="J35" s="3"/>
+      <c r="J35" s="3" t="s">
+        <v>101</v>
+      </c>
       <c r="K35" s="3"/>
-    </row>
-    <row r="36" spans="1:11">
+      <c r="N35" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15">
       <c r="A36" s="3"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
+      <c r="B36" s="3" t="str" cm="1">
+        <f t="array" ref="B36:B42">_xlfn.UNIQUE(B2:B31)</f>
+        <v>Ботинки</v>
+      </c>
+      <c r="C36" s="3">
+        <v>1</v>
+      </c>
       <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
+      <c r="E36" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F36" s="3">
+        <v>1</v>
+      </c>
+      <c r="G36" s="3" t="str" cm="1">
+        <f t="array" ref="G36:G37">_xlfn.UNIQUE(E2:E31)</f>
+        <v>Kari</v>
+      </c>
+      <c r="H36" s="3">
+        <v>1</v>
+      </c>
       <c r="I36" s="3"/>
-      <c r="J36" s="3"/>
-      <c r="K36" s="3"/>
-    </row>
-    <row r="37" spans="1:11">
+      <c r="J36" s="3" t="str" cm="1">
+        <f t="array" ref="J36:J37">_xlfn.UNIQUE(G2:G31)</f>
+        <v>Женская обувь</v>
+      </c>
+      <c r="K36" s="3">
+        <v>1</v>
+      </c>
+      <c r="N36" t="str" cm="1">
+        <f t="array" ref="N36:N41">_xlfn.UNIQUE(F2:F31)</f>
+        <v>Kari</v>
+      </c>
+      <c r="O36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15">
       <c r="A37" s="3"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
+      <c r="B37" s="3" t="str">
+        <v>Туфли</v>
+      </c>
+      <c r="C37" s="3">
+        <v>2</v>
+      </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
+      <c r="G37" s="3" t="str">
+        <v>Обувь для вас</v>
+      </c>
+      <c r="H37" s="3">
+        <v>2</v>
+      </c>
       <c r="I37" s="3"/>
-      <c r="J37" s="3"/>
-      <c r="K37" s="3"/>
-    </row>
-    <row r="38" spans="1:11">
+      <c r="J37" s="3" t="str">
+        <v>Мужская обувь</v>
+      </c>
+      <c r="K37" s="3">
+        <v>2</v>
+      </c>
+      <c r="N37" t="str">
+        <v>Marco Tozzi</v>
+      </c>
+      <c r="O37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15">
       <c r="A38" s="3"/>
-      <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
+      <c r="B38" s="3" t="str">
+        <v>Кроссовки</v>
+      </c>
+      <c r="C38" s="3">
+        <v>3</v>
+      </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
@@ -1854,11 +2209,21 @@
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
       <c r="K38" s="3"/>
-    </row>
-    <row r="39" spans="1:11">
+      <c r="N38" t="str">
+        <v>Рос</v>
+      </c>
+      <c r="O38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15">
       <c r="A39" s="3"/>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
+      <c r="B39" s="3" t="str">
+        <v>Полуботинки</v>
+      </c>
+      <c r="C39" s="3">
+        <v>4</v>
+      </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
@@ -1867,11 +2232,21 @@
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
-    </row>
-    <row r="40" spans="1:11">
+      <c r="N39" t="str">
+        <v>Rieker</v>
+      </c>
+      <c r="O39">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15">
       <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
+      <c r="B40" s="3" t="str">
+        <v>Кеды</v>
+      </c>
+      <c r="C40" s="3">
+        <v>5</v>
+      </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
@@ -1880,11 +2255,21 @@
       <c r="I40" s="3"/>
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
-    </row>
-    <row r="41" spans="1:11">
+      <c r="N40" t="str">
+        <v>Alessio Nesca</v>
+      </c>
+      <c r="O40">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15">
       <c r="A41" s="3"/>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
+      <c r="B41" s="3" t="str">
+        <v>Тапочки</v>
+      </c>
+      <c r="C41" s="3">
+        <v>6</v>
+      </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
@@ -1893,11 +2278,21 @@
       <c r="I41" s="3"/>
       <c r="J41" s="3"/>
       <c r="K41" s="3"/>
-    </row>
-    <row r="42" spans="1:11">
+      <c r="N41" t="str">
+        <v>CROSBY</v>
+      </c>
+      <c r="O41">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15">
       <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
+      <c r="B42" s="3" t="str">
+        <v>Сапоги</v>
+      </c>
+      <c r="C42" s="3">
+        <v>7</v>
+      </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
@@ -1907,7 +2302,7 @@
       <c r="J42" s="3"/>
       <c r="K42" s="3"/>
     </row>
-    <row r="43" spans="1:11">
+    <row r="43" spans="1:15">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
@@ -1920,7 +2315,7 @@
       <c r="J43" s="3"/>
       <c r="K43" s="3"/>
     </row>
-    <row r="44" spans="1:11">
+    <row r="44" spans="1:15">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -1933,8 +2328,1641 @@
       <c r="J44" s="3"/>
       <c r="K44" s="3"/>
     </row>
+    <row r="45" spans="1:15" ht="47.25">
+      <c r="A45">
+        <v>1</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C45" t="s">
+        <v>98</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H45" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J45" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K45" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" ht="31.5">
+      <c r="A46">
+        <v>2</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C46">
+        <f>VLOOKUP(B2,$B$36:$C$42,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="D46">
+        <v>1</v>
+      </c>
+      <c r="E46" s="11">
+        <v>1</v>
+      </c>
+      <c r="F46">
+        <f>VLOOKUP(F2,$N$36:$O$41,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="G46">
+        <f>VLOOKUP(G2,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H46" s="2">
+        <v>4990</v>
+      </c>
+      <c r="I46" s="2">
+        <v>3</v>
+      </c>
+      <c r="J46" s="2">
+        <v>6</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" ht="63">
+      <c r="A47">
+        <v>3</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C47">
+        <f>VLOOKUP(B3,$B$36:$C$42,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="D47">
+        <v>1</v>
+      </c>
+      <c r="E47" s="11">
+        <v>2</v>
+      </c>
+      <c r="F47">
+        <f>VLOOKUP(F3,$N$36:$O$41,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="G47">
+        <f>VLOOKUP(G3,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H47" s="2">
+        <v>3244</v>
+      </c>
+      <c r="I47" s="2">
+        <v>2</v>
+      </c>
+      <c r="J47" s="2">
+        <v>13</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" ht="63">
+      <c r="A48">
+        <v>4</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C48">
+        <f>VLOOKUP(B4,$B$36:$C$42,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="D48">
+        <v>1</v>
+      </c>
+      <c r="E48" s="11">
+        <v>1</v>
+      </c>
+      <c r="F48">
+        <f>VLOOKUP(F4,$N$36:$O$41,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="G48">
+        <f>VLOOKUP(G4,$J$36:$K$37,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="H48" s="2">
+        <v>4499</v>
+      </c>
+      <c r="I48" s="2">
+        <v>4</v>
+      </c>
+      <c r="J48" s="2">
+        <v>5</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="47.25">
+      <c r="A49">
+        <v>5</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C49">
+        <f>VLOOKUP(B5,$B$36:$C$42,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="D49">
+        <v>1</v>
+      </c>
+      <c r="E49" s="11">
+        <v>1</v>
+      </c>
+      <c r="F49">
+        <f>VLOOKUP(F5,$N$36:$O$41,2,FALSE)</f>
+        <v>3</v>
+      </c>
+      <c r="G49">
+        <f>VLOOKUP(G5,$J$36:$K$37,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="H49" s="2">
+        <v>5900</v>
+      </c>
+      <c r="I49" s="2">
+        <v>2</v>
+      </c>
+      <c r="J49" s="2">
+        <v>8</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="31.5">
+      <c r="A50">
+        <v>6</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C50">
+        <f>VLOOKUP(B6,$B$36:$C$42,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="D50">
+        <v>1</v>
+      </c>
+      <c r="E50" s="11">
+        <v>2</v>
+      </c>
+      <c r="F50">
+        <f>VLOOKUP(F6,$N$36:$O$41,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="G50">
+        <f>VLOOKUP(G6,$J$36:$K$37,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="H50" s="2">
+        <v>3800</v>
+      </c>
+      <c r="I50" s="2">
+        <v>2</v>
+      </c>
+      <c r="J50" s="2">
+        <v>16</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="31.5">
+      <c r="A51">
+        <v>7</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C51">
+        <f>VLOOKUP(B7,$B$36:$C$42,2,FALSE)</f>
+        <v>3</v>
+      </c>
+      <c r="D51">
+        <v>1</v>
+      </c>
+      <c r="E51" s="11">
+        <v>2</v>
+      </c>
+      <c r="F51">
+        <f>VLOOKUP(F7,$N$36:$O$41,2,FALSE)</f>
+        <v>3</v>
+      </c>
+      <c r="G51">
+        <f>VLOOKUP(G7,$J$36:$K$37,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="H51" s="2">
+        <v>4100</v>
+      </c>
+      <c r="I51" s="2">
+        <v>3</v>
+      </c>
+      <c r="J51" s="2">
+        <v>6</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="47.25">
+      <c r="A52">
+        <v>8</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C52">
+        <f>VLOOKUP(B8,$B$36:$C$42,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="D52">
+        <v>1</v>
+      </c>
+      <c r="E52" s="11">
+        <v>1</v>
+      </c>
+      <c r="F52">
+        <f>VLOOKUP(F8,$N$36:$O$41,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="G52">
+        <f>VLOOKUP(G8,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H52" s="2">
+        <v>2700</v>
+      </c>
+      <c r="I52" s="2">
+        <v>2</v>
+      </c>
+      <c r="J52" s="2">
+        <v>14</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="63">
+      <c r="A53">
+        <v>9</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C53">
+        <f>VLOOKUP(B9,$B$36:$C$42,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="D53">
+        <v>1</v>
+      </c>
+      <c r="E53" s="11">
+        <v>2</v>
+      </c>
+      <c r="F53">
+        <f>VLOOKUP(F9,$N$36:$O$41,2,FALSE)</f>
+        <v>5</v>
+      </c>
+      <c r="G53">
+        <f>VLOOKUP(G9,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H53" s="2">
+        <v>1890</v>
+      </c>
+      <c r="I53" s="2">
+        <v>4</v>
+      </c>
+      <c r="J53" s="2">
+        <v>4</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="47.25">
+      <c r="A54">
+        <v>10</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C54">
+        <f>VLOOKUP(B10,$B$36:$C$42,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
+      </c>
+      <c r="E54" s="11">
+        <v>1</v>
+      </c>
+      <c r="F54">
+        <f>VLOOKUP(F10,$N$36:$O$41,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="G54">
+        <f>VLOOKUP(G10,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H54" s="2">
+        <v>4300</v>
+      </c>
+      <c r="I54" s="2">
+        <v>2</v>
+      </c>
+      <c r="J54" s="2">
+        <v>6</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="47.25">
+      <c r="A55">
+        <v>11</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C55">
+        <f>VLOOKUP(B11,$B$36:$C$42,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="D55">
+        <v>1</v>
+      </c>
+      <c r="E55" s="11">
+        <v>1</v>
+      </c>
+      <c r="F55">
+        <f>VLOOKUP(F11,$N$36:$O$41,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="G55">
+        <f>VLOOKUP(G11,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H55" s="2">
+        <v>2800</v>
+      </c>
+      <c r="I55" s="2">
+        <v>3</v>
+      </c>
+      <c r="J55" s="2">
+        <v>15</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="47.25">
+      <c r="A56">
+        <v>12</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C56">
+        <f>VLOOKUP(B12,$B$36:$C$42,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="D56">
+        <v>1</v>
+      </c>
+      <c r="E56" s="11">
+        <v>2</v>
+      </c>
+      <c r="F56">
+        <f>VLOOKUP(F12,$N$36:$O$41,2,FALSE)</f>
+        <v>6</v>
+      </c>
+      <c r="G56">
+        <f>VLOOKUP(G12,$J$36:$K$37,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="H56" s="2">
+        <v>2156</v>
+      </c>
+      <c r="I56" s="2">
+        <v>3</v>
+      </c>
+      <c r="J56" s="2">
+        <v>6</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="47.25">
+      <c r="A57">
+        <v>13</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C57">
+        <f>VLOOKUP(B13,$B$36:$C$42,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="D57">
+        <v>1</v>
+      </c>
+      <c r="E57" s="11">
+        <v>1</v>
+      </c>
+      <c r="F57">
+        <f>VLOOKUP(F13,$N$36:$O$41,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="G57">
+        <f>VLOOKUP(G13,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H57" s="2">
+        <v>1800</v>
+      </c>
+      <c r="I57" s="2">
+        <v>2</v>
+      </c>
+      <c r="J57" s="2">
+        <v>14</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="47.25">
+      <c r="A58">
+        <v>14</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C58">
+        <f>VLOOKUP(B14,$B$36:$C$42,2,FALSE)</f>
+        <v>5</v>
+      </c>
+      <c r="D58">
+        <v>1</v>
+      </c>
+      <c r="E58" s="11">
+        <v>2</v>
+      </c>
+      <c r="F58">
+        <f>VLOOKUP(F14,$N$36:$O$41,2,FALSE)</f>
+        <v>6</v>
+      </c>
+      <c r="G58">
+        <f>VLOOKUP(G14,$J$36:$K$37,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="H58" s="2">
+        <v>5500</v>
+      </c>
+      <c r="I58" s="2">
+        <v>3</v>
+      </c>
+      <c r="J58" s="2">
+        <v>0</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="47.25">
+      <c r="A59">
+        <v>15</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C59">
+        <f>VLOOKUP(B15,$B$36:$C$42,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="D59">
+        <v>1</v>
+      </c>
+      <c r="E59" s="11">
+        <v>2</v>
+      </c>
+      <c r="F59">
+        <f>VLOOKUP(F15,$N$36:$O$41,2,FALSE)</f>
+        <v>6</v>
+      </c>
+      <c r="G59">
+        <f>VLOOKUP(G15,$J$36:$K$37,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="H59" s="2">
+        <v>2100</v>
+      </c>
+      <c r="I59" s="2">
+        <v>2</v>
+      </c>
+      <c r="J59" s="2">
+        <v>3</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="47.25">
+      <c r="A60">
+        <v>16</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C60">
+        <f>VLOOKUP(B16,$B$36:$C$42,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="D60">
+        <v>1</v>
+      </c>
+      <c r="E60" s="11">
+        <v>2</v>
+      </c>
+      <c r="F60">
+        <f>VLOOKUP(F16,$N$36:$O$41,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="G60">
+        <f>VLOOKUP(G16,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H60" s="2">
+        <v>5400</v>
+      </c>
+      <c r="I60" s="2">
+        <v>4</v>
+      </c>
+      <c r="J60" s="2">
+        <v>18</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="47.25">
+      <c r="A61">
+        <v>17</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C61">
+        <f>VLOOKUP(B17,$B$36:$C$42,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="D61">
+        <v>1</v>
+      </c>
+      <c r="E61" s="11">
+        <v>1</v>
+      </c>
+      <c r="F61">
+        <f>VLOOKUP(F17,$N$36:$O$41,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="G61">
+        <f>VLOOKUP(G17,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H61" s="2">
+        <v>6600</v>
+      </c>
+      <c r="I61" s="2">
+        <v>12</v>
+      </c>
+      <c r="J61" s="2">
+        <v>9</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="47.25">
+      <c r="A62">
+        <v>18</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C62">
+        <f>VLOOKUP(B18,$B$36:$C$42,2,FALSE)</f>
+        <v>6</v>
+      </c>
+      <c r="D62">
+        <v>1</v>
+      </c>
+      <c r="E62" s="11">
+        <v>1</v>
+      </c>
+      <c r="F62">
+        <f>VLOOKUP(F18,$N$36:$O$41,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="G62">
+        <f>VLOOKUP(G18,$J$36:$K$37,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="H62" s="2">
+        <v>500</v>
+      </c>
+      <c r="I62" s="2">
+        <v>13</v>
+      </c>
+      <c r="J62" s="2">
+        <v>0</v>
+      </c>
+      <c r="K62" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="47.25">
+      <c r="A63">
+        <v>19</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C63">
+        <f>VLOOKUP(B19,$B$36:$C$42,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="D63">
+        <v>1</v>
+      </c>
+      <c r="E63" s="11">
+        <v>2</v>
+      </c>
+      <c r="F63">
+        <f>VLOOKUP(F19,$N$36:$O$41,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="G63">
+        <f>VLOOKUP(G19,$J$36:$K$37,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="H63" s="2">
+        <v>2700</v>
+      </c>
+      <c r="I63" s="2">
+        <v>2</v>
+      </c>
+      <c r="J63" s="2">
+        <v>5</v>
+      </c>
+      <c r="K63" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="31.5">
+      <c r="A64">
+        <v>20</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C64">
+        <f>VLOOKUP(B20,$B$36:$C$42,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="D64">
+        <v>1</v>
+      </c>
+      <c r="E64" s="11">
+        <v>1</v>
+      </c>
+      <c r="F64">
+        <f>VLOOKUP(F20,$N$36:$O$41,2,FALSE)</f>
+        <v>6</v>
+      </c>
+      <c r="G64">
+        <f>VLOOKUP(G20,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H64" s="2">
+        <v>6800</v>
+      </c>
+      <c r="I64" s="2">
+        <v>15</v>
+      </c>
+      <c r="J64" s="2">
+        <v>15</v>
+      </c>
+      <c r="K64" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" ht="31.5">
+      <c r="A65">
+        <v>21</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C65">
+        <f>VLOOKUP(B21,$B$36:$C$42,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="D65">
+        <v>1</v>
+      </c>
+      <c r="E65" s="11">
+        <v>1</v>
+      </c>
+      <c r="F65">
+        <f>VLOOKUP(F21,$N$36:$O$41,2,FALSE)</f>
+        <v>5</v>
+      </c>
+      <c r="G65">
+        <f>VLOOKUP(G21,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H65" s="2">
+        <v>10200</v>
+      </c>
+      <c r="I65" s="2">
+        <v>15</v>
+      </c>
+      <c r="J65" s="2">
+        <v>9</v>
+      </c>
+      <c r="K65" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="47.25">
+      <c r="A66">
+        <v>22</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C66">
+        <f>VLOOKUP(B22,$B$36:$C$42,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="D66">
+        <v>1</v>
+      </c>
+      <c r="E66" s="11">
+        <v>2</v>
+      </c>
+      <c r="F66">
+        <f>VLOOKUP(F22,$N$36:$O$41,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="G66">
+        <f>VLOOKUP(G22,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H66" s="2">
+        <v>11800</v>
+      </c>
+      <c r="I66" s="2">
+        <v>15</v>
+      </c>
+      <c r="J66" s="2">
+        <v>11</v>
+      </c>
+      <c r="K66" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" ht="31.5">
+      <c r="A67">
+        <v>23</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C67">
+        <f>VLOOKUP(B23,$B$36:$C$42,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="D67">
+        <v>1</v>
+      </c>
+      <c r="E67" s="11">
+        <v>1</v>
+      </c>
+      <c r="F67">
+        <f>VLOOKUP(F23,$N$36:$O$41,2,FALSE)</f>
+        <v>6</v>
+      </c>
+      <c r="G67">
+        <f>VLOOKUP(G23,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H67" s="2">
+        <v>4600</v>
+      </c>
+      <c r="I67" s="2">
+        <v>3</v>
+      </c>
+      <c r="J67" s="2">
+        <v>13</v>
+      </c>
+      <c r="K67" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" ht="63">
+      <c r="A68">
+        <v>24</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C68">
+        <f>VLOOKUP(B24,$B$36:$C$42,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="D68">
+        <v>1</v>
+      </c>
+      <c r="E68" s="11">
+        <v>1</v>
+      </c>
+      <c r="F68">
+        <f>VLOOKUP(F24,$N$36:$O$41,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="G68">
+        <f>VLOOKUP(G24,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H68" s="2">
+        <v>12400</v>
+      </c>
+      <c r="I68" s="2">
+        <v>16</v>
+      </c>
+      <c r="J68" s="2">
+        <v>5</v>
+      </c>
+      <c r="K68" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" ht="47.25">
+      <c r="A69">
+        <v>25</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C69">
+        <f>VLOOKUP(B25,$B$36:$C$42,2,FALSE)</f>
+        <v>6</v>
+      </c>
+      <c r="D69">
+        <v>1</v>
+      </c>
+      <c r="E69" s="11">
+        <v>2</v>
+      </c>
+      <c r="F69">
+        <f>VLOOKUP(F25,$N$36:$O$41,2,FALSE)</f>
+        <v>6</v>
+      </c>
+      <c r="G69">
+        <f>VLOOKUP(G25,$J$36:$K$37,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="H69" s="2">
+        <v>9900</v>
+      </c>
+      <c r="I69" s="2">
+        <v>17</v>
+      </c>
+      <c r="J69" s="2">
+        <v>15</v>
+      </c>
+      <c r="K69" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" ht="47.25">
+      <c r="A70">
+        <v>26</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C70">
+        <f>VLOOKUP(B26,$B$36:$C$42,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="D70">
+        <v>1</v>
+      </c>
+      <c r="E70" s="11">
+        <v>1</v>
+      </c>
+      <c r="F70">
+        <f>VLOOKUP(F26,$N$36:$O$41,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="G70">
+        <f>VLOOKUP(G26,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H70" s="2">
+        <v>1700</v>
+      </c>
+      <c r="I70" s="2">
+        <v>2</v>
+      </c>
+      <c r="J70" s="2">
+        <v>7</v>
+      </c>
+      <c r="K70" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" ht="31.5">
+      <c r="A71">
+        <v>27</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C71">
+        <f>VLOOKUP(B27,$B$36:$C$42,2,FALSE)</f>
+        <v>3</v>
+      </c>
+      <c r="D71">
+        <v>1</v>
+      </c>
+      <c r="E71" s="11">
+        <v>2</v>
+      </c>
+      <c r="F71">
+        <f>VLOOKUP(F27,$N$36:$O$41,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="G71">
+        <f>VLOOKUP(G27,$J$36:$K$37,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="H71" s="2">
+        <v>2800</v>
+      </c>
+      <c r="I71" s="2">
+        <v>18</v>
+      </c>
+      <c r="J71" s="2">
+        <v>3</v>
+      </c>
+      <c r="K71" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" ht="47.25">
+      <c r="A72">
+        <v>28</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C72">
+        <f>VLOOKUP(B28,$B$36:$C$42,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="D72">
+        <v>1</v>
+      </c>
+      <c r="E72" s="11">
+        <v>2</v>
+      </c>
+      <c r="F72">
+        <f>VLOOKUP(F28,$N$36:$O$41,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="G72">
+        <f>VLOOKUP(G28,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H72" s="2">
+        <v>4399</v>
+      </c>
+      <c r="I72" s="2">
+        <v>3</v>
+      </c>
+      <c r="J72" s="2">
+        <v>12</v>
+      </c>
+      <c r="K72" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" ht="31.5">
+      <c r="A73">
+        <v>29</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C73">
+        <f>VLOOKUP(B29,$B$36:$C$42,2,FALSE)</f>
+        <v>7</v>
+      </c>
+      <c r="D73">
+        <v>1</v>
+      </c>
+      <c r="E73" s="11">
+        <v>1</v>
+      </c>
+      <c r="F73">
+        <f>VLOOKUP(F29,$N$36:$O$41,2,FALSE)</f>
+        <v>6</v>
+      </c>
+      <c r="G73">
+        <f>VLOOKUP(G29,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H73" s="2">
+        <v>4699</v>
+      </c>
+      <c r="I73" s="2">
+        <v>2</v>
+      </c>
+      <c r="J73" s="2">
+        <v>5</v>
+      </c>
+      <c r="K73" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" ht="31.5">
+      <c r="A74">
+        <v>30</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C74">
+        <f>VLOOKUP(B30,$B$36:$C$42,2,FALSE)</f>
+        <v>6</v>
+      </c>
+      <c r="D74">
+        <v>1</v>
+      </c>
+      <c r="E74" s="11">
+        <v>1</v>
+      </c>
+      <c r="F74">
+        <f>VLOOKUP(F30,$N$36:$O$41,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="G74">
+        <f>VLOOKUP(G30,$J$36:$K$37,2,FALSE)</f>
+        <v>2</v>
+      </c>
+      <c r="H74" s="2">
+        <v>599</v>
+      </c>
+      <c r="I74" s="2">
+        <v>20</v>
+      </c>
+      <c r="J74" s="2">
+        <v>2</v>
+      </c>
+      <c r="K74" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" ht="31.5">
+      <c r="A75">
+        <v>31</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C75">
+        <f>VLOOKUP(B31,$B$36:$C$42,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="D75">
+        <v>1</v>
+      </c>
+      <c r="E75" s="11">
+        <v>2</v>
+      </c>
+      <c r="F75">
+        <f>VLOOKUP(F31,$N$36:$O$41,2,FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="G75">
+        <f>VLOOKUP(G31,$J$36:$K$37,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="H75" s="2">
+        <v>2300</v>
+      </c>
+      <c r="I75" s="2">
+        <v>2</v>
+      </c>
+      <c r="J75" s="2">
+        <v>7</v>
+      </c>
+      <c r="K75" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{015D80BC-A256-44F2-9684-BB69A63D1C79}">
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="1" width="25.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="G2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="G3" t="str" cm="1">
+        <f t="array" ref="G3:G5">_xlfn.UNIQUE(A2:A11)</f>
+        <v>Администратор</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Менеджер</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Авторизированный клиент</v>
+      </c>
+      <c r="H5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C14" t="s">
+        <v>139</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15">
+        <f>VLOOKUP(A2,$G$3:$H$5,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16">
+        <f t="shared" ref="A16:A24" si="0">VLOOKUP(A3,$G$3:$H$5,2,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>136</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{08968244-D571-496D-A71A-270AEF16C785}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{3D909DD1-23EA-4261-889C-FF7BB3FED8F6}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{A7832D16-B200-4652-AF14-427362D2C9EA}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{1F85D63D-76AF-4082-82BA-72C82170DEA0}"/>
+    <hyperlink ref="C6" r:id="rId5" xr:uid="{FC31619C-27BA-4B3B-9C37-89B3EA3E6A96}"/>
+    <hyperlink ref="C7" r:id="rId6" xr:uid="{2CC64915-795F-4882-B96E-7B2FC00600F1}"/>
+    <hyperlink ref="C8" r:id="rId7" xr:uid="{B7CA4B9F-34AC-41D3-A108-18FADF264846}"/>
+    <hyperlink ref="C9" r:id="rId8" xr:uid="{4E7D3C41-0889-45B8-88C7-47BD438E3CEC}"/>
+    <hyperlink ref="C10" r:id="rId9" xr:uid="{85C85BB0-7BD0-48A4-AB1E-5C4AD80B3A0B}"/>
+    <hyperlink ref="C11" r:id="rId10" xr:uid="{97BA6185-252F-42F6-B8A8-2A13EB8B32C6}"/>
+    <hyperlink ref="E15" r:id="rId11" xr:uid="{FDEBB1DA-55AA-4682-8072-1B9E3DFE66E4}"/>
+    <hyperlink ref="E16" r:id="rId12" xr:uid="{F8111361-9610-4F6B-B00C-9058E54CF50B}"/>
+    <hyperlink ref="E17" r:id="rId13" xr:uid="{9A956D6A-0A79-41F3-8242-50EF385835D8}"/>
+    <hyperlink ref="E18" r:id="rId14" xr:uid="{A73B233B-26C0-47D6-846C-44CDBDAD58F3}"/>
+    <hyperlink ref="E19" r:id="rId15" xr:uid="{E4A23FE5-474F-4096-BE6F-D51F5CD7605E}"/>
+    <hyperlink ref="E20" r:id="rId16" xr:uid="{CF2ACE5B-4788-42C3-8BD8-4D2B1749CF91}"/>
+    <hyperlink ref="E21" r:id="rId17" xr:uid="{4F79D94E-76D5-4A8F-A881-70E792B84002}"/>
+    <hyperlink ref="E22" r:id="rId18" xr:uid="{57708CE7-F9D1-4A1B-9716-2FAF95A8811B}"/>
+    <hyperlink ref="E23" r:id="rId19" xr:uid="{3F089089-34F2-43C1-84F5-97553FF92C16}"/>
+    <hyperlink ref="E24" r:id="rId20" xr:uid="{A361FF70-71E6-45B3-9974-5F7ABF6C5703}"/>
+    <hyperlink ref="C15" r:id="rId21" display="mailto:94d5ous@gmail.com" xr:uid="{50C6A0A3-B779-4696-8A4B-B95B41620EE9}"/>
+    <hyperlink ref="C16" r:id="rId22" display="mailto:uth4iz@mail.com" xr:uid="{704F889A-11AC-4663-807B-98CE27170326}"/>
+    <hyperlink ref="C17" r:id="rId23" display="mailto:yzls62@outlook.com" xr:uid="{E31B6370-07EF-4BE4-94BC-345EBF0D05F8}"/>
+    <hyperlink ref="C18" r:id="rId24" display="mailto:1diph5e@tutanota.com" xr:uid="{AB9987AA-4366-42E3-B0FD-CAEB40DCA694}"/>
+    <hyperlink ref="C19" r:id="rId25" display="mailto:tjde7c@yahoo.com" xr:uid="{9D463F06-2B9C-4EC6-86A3-33E2518CDBF5}"/>
+    <hyperlink ref="C20" r:id="rId26" display="mailto:wpmrc3do@tutanota.com" xr:uid="{D49B38DE-6996-4FD3-9BF5-D769A611A3DB}"/>
+    <hyperlink ref="C21" r:id="rId27" display="mailto:5d4zbu@tutanota.com" xr:uid="{54EA3066-CE83-4071-924E-1E495F6C3C0E}"/>
+    <hyperlink ref="C22" r:id="rId28" display="mailto:ptec8ym@yahoo.com" xr:uid="{B260E1B3-BC05-46DE-B9FE-1EA5669207F7}"/>
+    <hyperlink ref="C23" r:id="rId29" display="mailto:1qz4kw@mail.com" xr:uid="{9B2EA303-4BCC-421B-AB48-32848026AD70}"/>
+    <hyperlink ref="C24" r:id="rId30" display="mailto:4np6se@mail.com" xr:uid="{217AEDE7-C7A1-4440-A5E7-C97A6A953A81}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId31"/>
+</worksheet>
 </file>
</xml_diff>